<commit_message>
Replace sample metadata with privacy-cleaned workbook
</commit_message>
<xml_diff>
--- a/metadata/Sample_metadata.xlsx
+++ b/metadata/Sample_metadata.xlsx
@@ -3,8 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20337"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15"/>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64FF1E6F-CF37-4FF0-AAF6-C1FB3F2B9B90}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="11520"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sample_metadata" sheetId="1" r:id="rId1"/>
@@ -3328,7 +3332,7 @@
         <v>61</v>
       </c>
       <c r="S14" s="6">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="T14" s="2" t="s">
         <v>62</v>
@@ -3382,7 +3386,7 @@
         <v>64</v>
       </c>
       <c r="S15" s="6">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="T15" s="2" t="s">
         <v>65</v>
@@ -3436,7 +3440,7 @@
         <v>67</v>
       </c>
       <c r="S16" s="6">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="T16" s="2" t="s">
         <v>68</v>
@@ -3490,7 +3494,7 @@
         <v>70</v>
       </c>
       <c r="S17" s="6">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="T17" s="2" t="s">
         <v>71</v>
@@ -3544,7 +3548,7 @@
         <v>73</v>
       </c>
       <c r="S18" s="6">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T18" s="2" t="s">
         <v>74</v>
@@ -3598,7 +3602,7 @@
         <v>76</v>
       </c>
       <c r="S19" s="6">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="T19" s="2" t="s">
         <v>77</v>
@@ -4360,7 +4364,7 @@
         <v>45</v>
       </c>
       <c r="S33" s="6">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="T33" s="2" t="s">
         <v>126</v>
@@ -4420,7 +4424,7 @@
         <v>46</v>
       </c>
       <c r="S34" s="6">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="T34" s="2" t="s">
         <v>129</v>
@@ -4480,7 +4484,7 @@
         <v>47</v>
       </c>
       <c r="S35" s="6">
-        <v>9</v>
+        <v>52</v>
       </c>
       <c r="T35" s="2" t="s">
         <v>132</v>
@@ -4540,7 +4544,7 @@
         <v>48</v>
       </c>
       <c r="S36" s="6">
-        <v>10</v>
+        <v>53</v>
       </c>
       <c r="T36" s="2" t="s">
         <v>135</v>
@@ -4594,7 +4598,7 @@
         <v>89</v>
       </c>
       <c r="S37" s="6">
-        <v>11</v>
+        <v>98</v>
       </c>
       <c r="T37" s="2" t="s">
         <v>140</v>
@@ -4648,7 +4652,7 @@
         <v>90</v>
       </c>
       <c r="S38" s="6">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="T38" s="2" t="s">
         <v>143</v>
@@ -4702,7 +4706,7 @@
         <v>91</v>
       </c>
       <c r="S39" s="6">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="T39" s="2" t="s">
         <v>146</v>
@@ -4756,7 +4760,7 @@
         <v>92</v>
       </c>
       <c r="S40" s="6">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="T40" s="2" t="s">
         <v>149</v>
@@ -4816,7 +4820,7 @@
         <v>133</v>
       </c>
       <c r="S41" s="6">
-        <v>16</v>
+        <v>146</v>
       </c>
       <c r="T41" s="2" t="s">
         <v>154</v>
@@ -4876,7 +4880,7 @@
         <v>134</v>
       </c>
       <c r="S42" s="6">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="T42" s="2" t="s">
         <v>157</v>
@@ -4936,7 +4940,7 @@
         <v>135</v>
       </c>
       <c r="S43" s="6">
-        <v>17</v>
+        <v>148</v>
       </c>
       <c r="T43" s="2" t="s">
         <v>160</v>
@@ -4996,7 +5000,7 @@
         <v>136</v>
       </c>
       <c r="S44" s="6">
-        <v>27</v>
+        <v>149</v>
       </c>
       <c r="T44" s="2" t="s">
         <v>163</v>
@@ -5056,7 +5060,7 @@
         <v>177</v>
       </c>
       <c r="S45" s="6">
-        <v>25</v>
+        <v>193</v>
       </c>
       <c r="T45" s="2" t="s">
         <v>168</v>
@@ -5116,7 +5120,7 @@
         <v>178</v>
       </c>
       <c r="S46" s="6">
-        <v>22</v>
+        <v>194</v>
       </c>
       <c r="T46" s="2" t="s">
         <v>171</v>
@@ -5176,7 +5180,7 @@
         <v>179</v>
       </c>
       <c r="S47" s="6">
-        <v>23</v>
+        <v>195</v>
       </c>
       <c r="T47" s="2" t="s">
         <v>174</v>
@@ -5236,7 +5240,7 @@
         <v>180</v>
       </c>
       <c r="S48" s="6">
-        <v>24</v>
+        <v>196</v>
       </c>
       <c r="T48" s="2" t="s">
         <v>177</v>
@@ -5298,7 +5302,7 @@
         <v>221</v>
       </c>
       <c r="S49" s="6">
-        <v>18</v>
+        <v>241</v>
       </c>
       <c r="T49" s="2" t="s">
         <v>182</v>
@@ -5360,7 +5364,7 @@
         <v>222</v>
       </c>
       <c r="S50" s="6">
-        <v>19</v>
+        <v>242</v>
       </c>
       <c r="T50" s="2" t="s">
         <v>185</v>
@@ -5422,7 +5426,7 @@
         <v>223</v>
       </c>
       <c r="S51" s="6">
-        <v>20</v>
+        <v>243</v>
       </c>
       <c r="T51" s="2" t="s">
         <v>188</v>
@@ -5484,7 +5488,7 @@
         <v>224</v>
       </c>
       <c r="S52" s="6">
-        <v>21</v>
+        <v>244</v>
       </c>
       <c r="T52" s="2" t="s">
         <v>191</v>
@@ -5538,7 +5542,7 @@
         <v>5</v>
       </c>
       <c r="S53" s="6">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="T53" s="2" t="s">
         <v>195</v>
@@ -5592,7 +5596,7 @@
         <v>6</v>
       </c>
       <c r="S54" s="6">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="T54" s="2" t="s">
         <v>197</v>
@@ -5646,7 +5650,7 @@
         <v>7</v>
       </c>
       <c r="S55" s="6">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="T55" s="2" t="s">
         <v>199</v>
@@ -5700,7 +5704,7 @@
         <v>8</v>
       </c>
       <c r="S56" s="6">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="T56" s="2" t="s">
         <v>201</v>
@@ -5760,7 +5764,7 @@
         <v>49</v>
       </c>
       <c r="S57" s="6">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="T57" s="2" t="s">
         <v>203</v>
@@ -5820,7 +5824,7 @@
         <v>50</v>
       </c>
       <c r="S58" s="6">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="T58" s="2" t="s">
         <v>205</v>
@@ -5880,7 +5884,7 @@
         <v>51</v>
       </c>
       <c r="S59" s="6">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="T59" s="2" t="s">
         <v>207</v>
@@ -5940,7 +5944,7 @@
         <v>52</v>
       </c>
       <c r="S60" s="6">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="T60" s="2" t="s">
         <v>209</v>
@@ -5994,7 +5998,7 @@
         <v>93</v>
       </c>
       <c r="S61" s="6">
-        <v>37</v>
+        <v>102</v>
       </c>
       <c r="T61" s="2" t="s">
         <v>211</v>
@@ -6048,7 +6052,7 @@
         <v>94</v>
       </c>
       <c r="S62" s="6">
-        <v>38</v>
+        <v>103</v>
       </c>
       <c r="T62" s="2" t="s">
         <v>213</v>
@@ -6102,7 +6106,7 @@
         <v>95</v>
       </c>
       <c r="S63" s="6">
-        <v>39</v>
+        <v>104</v>
       </c>
       <c r="T63" s="2" t="s">
         <v>215</v>
@@ -6156,7 +6160,7 @@
         <v>96</v>
       </c>
       <c r="S64" s="6">
-        <v>40</v>
+        <v>105</v>
       </c>
       <c r="T64" s="2" t="s">
         <v>217</v>
@@ -6216,7 +6220,7 @@
         <v>137</v>
       </c>
       <c r="S65" s="6">
-        <v>42</v>
+        <v>150</v>
       </c>
       <c r="T65" s="2" t="s">
         <v>219</v>
@@ -6276,7 +6280,7 @@
         <v>138</v>
       </c>
       <c r="S66" s="6">
-        <v>43</v>
+        <v>151</v>
       </c>
       <c r="T66" s="2" t="s">
         <v>221</v>
@@ -6336,7 +6340,7 @@
         <v>139</v>
       </c>
       <c r="S67" s="6">
-        <v>44</v>
+        <v>152</v>
       </c>
       <c r="T67" s="2" t="s">
         <v>223</v>
@@ -6396,7 +6400,7 @@
         <v>140</v>
       </c>
       <c r="S68" s="6">
-        <v>45</v>
+        <v>153</v>
       </c>
       <c r="T68" s="2" t="s">
         <v>225</v>
@@ -6456,7 +6460,7 @@
         <v>181</v>
       </c>
       <c r="S69" s="6">
-        <v>46</v>
+        <v>198</v>
       </c>
       <c r="T69" s="2" t="s">
         <v>227</v>
@@ -6516,7 +6520,7 @@
         <v>182</v>
       </c>
       <c r="S70" s="6">
-        <v>47</v>
+        <v>199</v>
       </c>
       <c r="T70" s="2" t="s">
         <v>229</v>
@@ -6576,7 +6580,7 @@
         <v>183</v>
       </c>
       <c r="S71" s="6">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="T71" s="2" t="s">
         <v>231</v>
@@ -6636,7 +6640,7 @@
         <v>184</v>
       </c>
       <c r="S72" s="6">
-        <v>49</v>
+        <v>201</v>
       </c>
       <c r="T72" s="2" t="s">
         <v>233</v>
@@ -6698,7 +6702,7 @@
         <v>225</v>
       </c>
       <c r="S73" s="6">
-        <v>50</v>
+        <v>245</v>
       </c>
       <c r="T73" s="2" t="s">
         <v>235</v>
@@ -6760,7 +6764,7 @@
         <v>226</v>
       </c>
       <c r="S74" s="6">
-        <v>51</v>
+        <v>246</v>
       </c>
       <c r="T74" s="2" t="s">
         <v>237</v>
@@ -6822,7 +6826,7 @@
         <v>227</v>
       </c>
       <c r="S75" s="6">
-        <v>52</v>
+        <v>247</v>
       </c>
       <c r="T75" s="2" t="s">
         <v>239</v>
@@ -6884,7 +6888,7 @@
         <v>228</v>
       </c>
       <c r="S76" s="6">
-        <v>53</v>
+        <v>248</v>
       </c>
       <c r="T76" s="2" t="s">
         <v>241</v>
@@ -6938,7 +6942,7 @@
         <v>9</v>
       </c>
       <c r="S77" s="6">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="T77" s="2" t="s">
         <v>245</v>
@@ -6992,7 +6996,7 @@
         <v>10</v>
       </c>
       <c r="S78" s="6">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="T78" s="2" t="s">
         <v>247</v>
@@ -7046,7 +7050,7 @@
         <v>11</v>
       </c>
       <c r="S79" s="6">
-        <v>57</v>
+        <v>13</v>
       </c>
       <c r="T79" s="2" t="s">
         <v>249</v>
@@ -7100,7 +7104,7 @@
         <v>12</v>
       </c>
       <c r="S80" s="6">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="T80" s="2" t="s">
         <v>251</v>
@@ -7394,7 +7398,7 @@
         <v>97</v>
       </c>
       <c r="S85" s="6">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="T85" s="2" t="s">
         <v>261</v>
@@ -7448,7 +7452,7 @@
         <v>98</v>
       </c>
       <c r="S86" s="6">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="T86" s="2" t="s">
         <v>263</v>
@@ -7502,7 +7506,7 @@
         <v>99</v>
       </c>
       <c r="S87" s="6">
-        <v>65</v>
+        <v>109</v>
       </c>
       <c r="T87" s="2" t="s">
         <v>265</v>
@@ -7556,7 +7560,7 @@
         <v>100</v>
       </c>
       <c r="S88" s="6">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="T88" s="2" t="s">
         <v>267</v>
@@ -7616,7 +7620,7 @@
         <v>141</v>
       </c>
       <c r="S89" s="6">
-        <v>72</v>
+        <v>154</v>
       </c>
       <c r="T89" s="2" t="s">
         <v>269</v>
@@ -7676,7 +7680,7 @@
         <v>142</v>
       </c>
       <c r="S90" s="6">
-        <v>73</v>
+        <v>155</v>
       </c>
       <c r="T90" s="2" t="s">
         <v>271</v>
@@ -7736,7 +7740,7 @@
         <v>143</v>
       </c>
       <c r="S91" s="6">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="T91" s="2" t="s">
         <v>273</v>
@@ -7796,7 +7800,7 @@
         <v>144</v>
       </c>
       <c r="S92" s="6">
-        <v>75</v>
+        <v>157</v>
       </c>
       <c r="T92" s="2" t="s">
         <v>275</v>
@@ -7856,7 +7860,7 @@
         <v>185</v>
       </c>
       <c r="S93" s="6">
-        <v>76</v>
+        <v>202</v>
       </c>
       <c r="T93" s="2" t="s">
         <v>277</v>
@@ -7916,7 +7920,7 @@
         <v>186</v>
       </c>
       <c r="S94" s="6">
-        <v>77</v>
+        <v>203</v>
       </c>
       <c r="T94" s="2" t="s">
         <v>279</v>
@@ -7976,7 +7980,7 @@
         <v>187</v>
       </c>
       <c r="S95" s="6">
-        <v>78</v>
+        <v>204</v>
       </c>
       <c r="T95" s="2" t="s">
         <v>281</v>
@@ -8036,7 +8040,7 @@
         <v>188</v>
       </c>
       <c r="S96" s="6">
-        <v>79</v>
+        <v>205</v>
       </c>
       <c r="T96" s="2" t="s">
         <v>283</v>
@@ -8098,7 +8102,7 @@
         <v>229</v>
       </c>
       <c r="S97" s="6">
-        <v>68</v>
+        <v>250</v>
       </c>
       <c r="T97" s="2" t="s">
         <v>285</v>
@@ -8160,7 +8164,7 @@
         <v>230</v>
       </c>
       <c r="S98" s="6">
-        <v>69</v>
+        <v>251</v>
       </c>
       <c r="T98" s="2" t="s">
         <v>287</v>
@@ -8222,7 +8226,7 @@
         <v>231</v>
       </c>
       <c r="S99" s="6">
-        <v>70</v>
+        <v>252</v>
       </c>
       <c r="T99" s="2" t="s">
         <v>289</v>
@@ -8284,7 +8288,7 @@
         <v>232</v>
       </c>
       <c r="S100" s="6">
-        <v>71</v>
+        <v>253</v>
       </c>
       <c r="T100" s="2" t="s">
         <v>291</v>
@@ -8338,7 +8342,7 @@
         <v>13</v>
       </c>
       <c r="S101" s="6">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="T101" s="2" t="s">
         <v>295</v>
@@ -8392,7 +8396,7 @@
         <v>14</v>
       </c>
       <c r="S102" s="6">
-        <v>82</v>
+        <v>17</v>
       </c>
       <c r="T102" s="2" t="s">
         <v>297</v>
@@ -8446,7 +8450,7 @@
         <v>15</v>
       </c>
       <c r="S103" s="6">
-        <v>83</v>
+        <v>18</v>
       </c>
       <c r="T103" s="2" t="s">
         <v>299</v>
@@ -8500,7 +8504,7 @@
         <v>16</v>
       </c>
       <c r="S104" s="6">
-        <v>84</v>
+        <v>19</v>
       </c>
       <c r="T104" s="2" t="s">
         <v>301</v>
@@ -8560,7 +8564,7 @@
         <v>57</v>
       </c>
       <c r="S105" s="6">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="T105" s="2" t="s">
         <v>303</v>
@@ -8620,7 +8624,7 @@
         <v>58</v>
       </c>
       <c r="S106" s="6">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="T106" s="2" t="s">
         <v>305</v>
@@ -8680,7 +8684,7 @@
         <v>59</v>
       </c>
       <c r="S107" s="6">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="T107" s="2" t="s">
         <v>307</v>
@@ -8740,7 +8744,7 @@
         <v>60</v>
       </c>
       <c r="S108" s="6">
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="T108" s="2" t="s">
         <v>309</v>
@@ -8794,7 +8798,7 @@
         <v>101</v>
       </c>
       <c r="S109" s="6">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="T109" s="2" t="s">
         <v>311</v>
@@ -8848,7 +8852,7 @@
         <v>102</v>
       </c>
       <c r="S110" s="6">
-        <v>90</v>
+        <v>112</v>
       </c>
       <c r="T110" s="2" t="s">
         <v>313</v>
@@ -8902,7 +8906,7 @@
         <v>103</v>
       </c>
       <c r="S111" s="6">
-        <v>91</v>
+        <v>113</v>
       </c>
       <c r="T111" s="2" t="s">
         <v>315</v>
@@ -8956,7 +8960,7 @@
         <v>104</v>
       </c>
       <c r="S112" s="6">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="T112" s="2" t="s">
         <v>317</v>
@@ -9016,7 +9020,7 @@
         <v>145</v>
       </c>
       <c r="S113" s="6">
-        <v>94</v>
+        <v>159</v>
       </c>
       <c r="T113" s="2" t="s">
         <v>319</v>
@@ -9076,7 +9080,7 @@
         <v>146</v>
       </c>
       <c r="S114" s="6">
-        <v>95</v>
+        <v>160</v>
       </c>
       <c r="T114" s="2" t="s">
         <v>321</v>
@@ -9136,7 +9140,7 @@
         <v>147</v>
       </c>
       <c r="S115" s="6">
-        <v>96</v>
+        <v>161</v>
       </c>
       <c r="T115" s="2" t="s">
         <v>323</v>
@@ -9196,7 +9200,7 @@
         <v>148</v>
       </c>
       <c r="S116" s="6">
-        <v>97</v>
+        <v>162</v>
       </c>
       <c r="T116" s="2" t="s">
         <v>325</v>
@@ -9256,7 +9260,7 @@
         <v>189</v>
       </c>
       <c r="S117" s="6">
-        <v>98</v>
+        <v>206</v>
       </c>
       <c r="T117" s="2" t="s">
         <v>327</v>
@@ -9316,7 +9320,7 @@
         <v>190</v>
       </c>
       <c r="S118" s="6">
-        <v>99</v>
+        <v>207</v>
       </c>
       <c r="T118" s="2" t="s">
         <v>329</v>
@@ -9376,7 +9380,7 @@
         <v>191</v>
       </c>
       <c r="S119" s="6">
-        <v>100</v>
+        <v>208</v>
       </c>
       <c r="T119" s="2" t="s">
         <v>331</v>
@@ -9436,7 +9440,7 @@
         <v>192</v>
       </c>
       <c r="S120" s="6">
-        <v>101</v>
+        <v>209</v>
       </c>
       <c r="T120" s="2" t="s">
         <v>333</v>
@@ -9498,7 +9502,7 @@
         <v>233</v>
       </c>
       <c r="S121" s="6">
-        <v>102</v>
+        <v>254</v>
       </c>
       <c r="T121" s="2" t="s">
         <v>335</v>
@@ -9560,7 +9564,7 @@
         <v>234</v>
       </c>
       <c r="S122" s="6">
-        <v>103</v>
+        <v>255</v>
       </c>
       <c r="T122" s="2" t="s">
         <v>337</v>
@@ -9622,7 +9626,7 @@
         <v>235</v>
       </c>
       <c r="S123" s="6">
-        <v>104</v>
+        <v>256</v>
       </c>
       <c r="T123" s="2" t="s">
         <v>339</v>
@@ -9684,7 +9688,7 @@
         <v>236</v>
       </c>
       <c r="S124" s="6">
-        <v>105</v>
+        <v>257</v>
       </c>
       <c r="T124" s="2" t="s">
         <v>341</v>
@@ -9738,7 +9742,7 @@
         <v>17</v>
       </c>
       <c r="S125" s="6">
-        <v>107</v>
+        <v>20</v>
       </c>
       <c r="T125" s="2" t="s">
         <v>345</v>
@@ -9792,7 +9796,7 @@
         <v>18</v>
       </c>
       <c r="S126" s="6">
-        <v>108</v>
+        <v>21</v>
       </c>
       <c r="T126" s="2" t="s">
         <v>347</v>
@@ -9846,7 +9850,7 @@
         <v>19</v>
       </c>
       <c r="S127" s="6">
-        <v>109</v>
+        <v>22</v>
       </c>
       <c r="T127" s="2" t="s">
         <v>349</v>
@@ -9900,7 +9904,7 @@
         <v>20</v>
       </c>
       <c r="S128" s="6">
-        <v>110</v>
+        <v>23</v>
       </c>
       <c r="T128" s="2" t="s">
         <v>351</v>
@@ -9960,7 +9964,7 @@
         <v>61</v>
       </c>
       <c r="S129" s="6">
-        <v>111</v>
+        <v>68</v>
       </c>
       <c r="T129" s="2" t="s">
         <v>353</v>
@@ -10020,7 +10024,7 @@
         <v>62</v>
       </c>
       <c r="S130" s="6">
-        <v>112</v>
+        <v>69</v>
       </c>
       <c r="T130" s="2" t="s">
         <v>355</v>
@@ -10080,7 +10084,7 @@
         <v>63</v>
       </c>
       <c r="S131" s="6">
-        <v>113</v>
+        <v>70</v>
       </c>
       <c r="T131" s="2" t="s">
         <v>357</v>
@@ -10140,7 +10144,7 @@
         <v>64</v>
       </c>
       <c r="S132" s="6">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="T132" s="2" t="s">
         <v>359</v>
@@ -10356,7 +10360,7 @@
         <v>108</v>
       </c>
       <c r="S136" s="6">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="T136" s="2" t="s">
         <v>367</v>
@@ -10416,7 +10420,7 @@
         <v>149</v>
       </c>
       <c r="S137" s="6">
-        <v>121</v>
+        <v>163</v>
       </c>
       <c r="T137" s="2" t="s">
         <v>369</v>
@@ -10476,7 +10480,7 @@
         <v>150</v>
       </c>
       <c r="S138" s="6">
-        <v>122</v>
+        <v>164</v>
       </c>
       <c r="T138" s="2" t="s">
         <v>371</v>
@@ -10536,7 +10540,7 @@
         <v>151</v>
       </c>
       <c r="S139" s="6">
-        <v>123</v>
+        <v>165</v>
       </c>
       <c r="T139" s="2" t="s">
         <v>373</v>
@@ -10596,7 +10600,7 @@
         <v>152</v>
       </c>
       <c r="S140" s="6">
-        <v>124</v>
+        <v>166</v>
       </c>
       <c r="T140" s="2" t="s">
         <v>375</v>
@@ -10656,7 +10660,7 @@
         <v>193</v>
       </c>
       <c r="S141" s="6">
-        <v>125</v>
+        <v>211</v>
       </c>
       <c r="T141" s="2" t="s">
         <v>377</v>
@@ -10716,7 +10720,7 @@
         <v>194</v>
       </c>
       <c r="S142" s="6">
-        <v>126</v>
+        <v>212</v>
       </c>
       <c r="T142" s="2" t="s">
         <v>379</v>
@@ -10776,7 +10780,7 @@
         <v>195</v>
       </c>
       <c r="S143" s="6">
-        <v>127</v>
+        <v>213</v>
       </c>
       <c r="T143" s="2" t="s">
         <v>381</v>
@@ -10836,7 +10840,7 @@
         <v>196</v>
       </c>
       <c r="S144" s="6">
-        <v>128</v>
+        <v>214</v>
       </c>
       <c r="T144" s="2" t="s">
         <v>383</v>
@@ -10898,7 +10902,7 @@
         <v>237</v>
       </c>
       <c r="S145" s="6">
-        <v>129</v>
+        <v>258</v>
       </c>
       <c r="T145" s="2" t="s">
         <v>385</v>
@@ -10960,7 +10964,7 @@
         <v>238</v>
       </c>
       <c r="S146" s="6">
-        <v>130</v>
+        <v>259</v>
       </c>
       <c r="T146" s="2" t="s">
         <v>387</v>
@@ -11022,7 +11026,7 @@
         <v>239</v>
       </c>
       <c r="S147" s="6">
-        <v>131</v>
+        <v>260</v>
       </c>
       <c r="T147" s="2" t="s">
         <v>389</v>
@@ -11084,7 +11088,7 @@
         <v>240</v>
       </c>
       <c r="S148" s="6">
-        <v>132</v>
+        <v>261</v>
       </c>
       <c r="T148" s="2" t="s">
         <v>391</v>
@@ -11138,7 +11142,7 @@
         <v>21</v>
       </c>
       <c r="S149" s="6">
-        <v>134</v>
+        <v>24</v>
       </c>
       <c r="T149" s="2" t="s">
         <v>395</v>
@@ -11192,7 +11196,7 @@
         <v>22</v>
       </c>
       <c r="S150" s="6">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="T150" s="2" t="s">
         <v>397</v>
@@ -11246,7 +11250,7 @@
         <v>23</v>
       </c>
       <c r="S151" s="6">
-        <v>136</v>
+        <v>26</v>
       </c>
       <c r="T151" s="2" t="s">
         <v>399</v>
@@ -11300,7 +11304,7 @@
         <v>24</v>
       </c>
       <c r="S152" s="6">
-        <v>137</v>
+        <v>27</v>
       </c>
       <c r="T152" s="2" t="s">
         <v>401</v>
@@ -11360,7 +11364,7 @@
         <v>65</v>
       </c>
       <c r="S153" s="6">
-        <v>138</v>
+        <v>72</v>
       </c>
       <c r="T153" s="2" t="s">
         <v>403</v>
@@ -11420,7 +11424,7 @@
         <v>66</v>
       </c>
       <c r="S154" s="6">
-        <v>139</v>
+        <v>73</v>
       </c>
       <c r="T154" s="2" t="s">
         <v>405</v>
@@ -11480,7 +11484,7 @@
         <v>67</v>
       </c>
       <c r="S155" s="6">
-        <v>140</v>
+        <v>74</v>
       </c>
       <c r="T155" s="2" t="s">
         <v>407</v>
@@ -11540,7 +11544,7 @@
         <v>68</v>
       </c>
       <c r="S156" s="6">
-        <v>141</v>
+        <v>75</v>
       </c>
       <c r="T156" s="2" t="s">
         <v>409</v>
@@ -11594,7 +11598,7 @@
         <v>109</v>
       </c>
       <c r="S157" s="6">
-        <v>155</v>
+        <v>120</v>
       </c>
       <c r="T157" s="2" t="s">
         <v>411</v>
@@ -11648,7 +11652,7 @@
         <v>110</v>
       </c>
       <c r="S158" s="6">
-        <v>156</v>
+        <v>121</v>
       </c>
       <c r="T158" s="2" t="s">
         <v>413</v>
@@ -11702,7 +11706,7 @@
         <v>111</v>
       </c>
       <c r="S159" s="6">
-        <v>157</v>
+        <v>122</v>
       </c>
       <c r="T159" s="2" t="s">
         <v>415</v>
@@ -11756,7 +11760,7 @@
         <v>112</v>
       </c>
       <c r="S160" s="6">
-        <v>158</v>
+        <v>123</v>
       </c>
       <c r="T160" s="2" t="s">
         <v>417</v>
@@ -11816,7 +11820,7 @@
         <v>153</v>
       </c>
       <c r="S161" s="6">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="T161" s="2" t="s">
         <v>419</v>
@@ -11876,7 +11880,7 @@
         <v>154</v>
       </c>
       <c r="S162" s="6">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="T162" s="2" t="s">
         <v>421</v>
@@ -11936,7 +11940,7 @@
         <v>155</v>
       </c>
       <c r="S163" s="6">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="T163" s="2" t="s">
         <v>423</v>
@@ -11996,7 +12000,7 @@
         <v>156</v>
       </c>
       <c r="S164" s="6">
-        <v>146</v>
+        <v>170</v>
       </c>
       <c r="T164" s="2" t="s">
         <v>425</v>
@@ -12056,7 +12060,7 @@
         <v>197</v>
       </c>
       <c r="S165" s="6">
-        <v>147</v>
+        <v>215</v>
       </c>
       <c r="T165" s="2" t="s">
         <v>427</v>
@@ -12116,7 +12120,7 @@
         <v>198</v>
       </c>
       <c r="S166" s="6">
-        <v>148</v>
+        <v>216</v>
       </c>
       <c r="T166" s="2" t="s">
         <v>429</v>
@@ -12176,7 +12180,7 @@
         <v>199</v>
       </c>
       <c r="S167" s="6">
-        <v>149</v>
+        <v>217</v>
       </c>
       <c r="T167" s="2" t="s">
         <v>431</v>
@@ -12236,7 +12240,7 @@
         <v>200</v>
       </c>
       <c r="S168" s="6">
-        <v>150</v>
+        <v>218</v>
       </c>
       <c r="T168" s="2" t="s">
         <v>433</v>
@@ -12298,7 +12302,7 @@
         <v>241</v>
       </c>
       <c r="S169" s="6">
-        <v>151</v>
+        <v>263</v>
       </c>
       <c r="T169" s="2" t="s">
         <v>435</v>
@@ -12360,7 +12364,7 @@
         <v>242</v>
       </c>
       <c r="S170" s="6">
-        <v>152</v>
+        <v>264</v>
       </c>
       <c r="T170" s="2" t="s">
         <v>437</v>
@@ -12422,7 +12426,7 @@
         <v>243</v>
       </c>
       <c r="S171" s="6">
-        <v>153</v>
+        <v>265</v>
       </c>
       <c r="T171" s="2" t="s">
         <v>439</v>
@@ -12484,7 +12488,7 @@
         <v>244</v>
       </c>
       <c r="S172" s="6">
-        <v>154</v>
+        <v>266</v>
       </c>
       <c r="T172" s="2" t="s">
         <v>441</v>
@@ -12538,7 +12542,7 @@
         <v>25</v>
       </c>
       <c r="S173" s="6">
-        <v>160</v>
+        <v>29</v>
       </c>
       <c r="T173" s="2" t="s">
         <v>445</v>
@@ -12592,7 +12596,7 @@
         <v>26</v>
       </c>
       <c r="S174" s="6">
-        <v>161</v>
+        <v>30</v>
       </c>
       <c r="T174" s="2" t="s">
         <v>447</v>
@@ -12646,7 +12650,7 @@
         <v>27</v>
       </c>
       <c r="S175" s="6">
-        <v>162</v>
+        <v>31</v>
       </c>
       <c r="T175" s="2" t="s">
         <v>449</v>
@@ -12700,7 +12704,7 @@
         <v>28</v>
       </c>
       <c r="S176" s="6">
-        <v>163</v>
+        <v>32</v>
       </c>
       <c r="T176" s="2" t="s">
         <v>451</v>
@@ -12760,7 +12764,7 @@
         <v>69</v>
       </c>
       <c r="S177" s="6">
-        <v>164</v>
+        <v>76</v>
       </c>
       <c r="T177" s="2" t="s">
         <v>453</v>
@@ -12820,7 +12824,7 @@
         <v>70</v>
       </c>
       <c r="S178" s="6">
-        <v>165</v>
+        <v>77</v>
       </c>
       <c r="T178" s="2" t="s">
         <v>455</v>
@@ -12880,7 +12884,7 @@
         <v>71</v>
       </c>
       <c r="S179" s="6">
-        <v>166</v>
+        <v>78</v>
       </c>
       <c r="T179" s="2" t="s">
         <v>457</v>
@@ -12940,7 +12944,7 @@
         <v>72</v>
       </c>
       <c r="S180" s="6">
-        <v>167</v>
+        <v>79</v>
       </c>
       <c r="T180" s="2" t="s">
         <v>459</v>
@@ -12994,7 +12998,7 @@
         <v>113</v>
       </c>
       <c r="S181" s="6">
-        <v>168</v>
+        <v>124</v>
       </c>
       <c r="T181" s="2" t="s">
         <v>461</v>
@@ -13048,7 +13052,7 @@
         <v>114</v>
       </c>
       <c r="S182" s="6">
-        <v>169</v>
+        <v>125</v>
       </c>
       <c r="T182" s="2" t="s">
         <v>463</v>
@@ -13102,7 +13106,7 @@
         <v>115</v>
       </c>
       <c r="S183" s="6">
-        <v>170</v>
+        <v>126</v>
       </c>
       <c r="T183" s="2" t="s">
         <v>465</v>
@@ -13156,7 +13160,7 @@
         <v>116</v>
       </c>
       <c r="S184" s="6">
-        <v>171</v>
+        <v>127</v>
       </c>
       <c r="T184" s="2" t="s">
         <v>467</v>
@@ -13216,7 +13220,7 @@
         <v>157</v>
       </c>
       <c r="S185" s="6">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T185" s="2" t="s">
         <v>469</v>
@@ -13276,7 +13280,7 @@
         <v>158</v>
       </c>
       <c r="S186" s="6">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="T186" s="2" t="s">
         <v>471</v>
@@ -13336,7 +13340,7 @@
         <v>159</v>
       </c>
       <c r="S187" s="6">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T187" s="2" t="s">
         <v>473</v>
@@ -13396,7 +13400,7 @@
         <v>160</v>
       </c>
       <c r="S188" s="6">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T188" s="2" t="s">
         <v>475</v>
@@ -13456,7 +13460,7 @@
         <v>201</v>
       </c>
       <c r="S189" s="6">
-        <v>177</v>
+        <v>219</v>
       </c>
       <c r="T189" s="2" t="s">
         <v>477</v>
@@ -13516,7 +13520,7 @@
         <v>202</v>
       </c>
       <c r="S190" s="6">
-        <v>178</v>
+        <v>220</v>
       </c>
       <c r="T190" s="2" t="s">
         <v>479</v>
@@ -13576,7 +13580,7 @@
         <v>203</v>
       </c>
       <c r="S191" s="6">
-        <v>179</v>
+        <v>221</v>
       </c>
       <c r="T191" s="2" t="s">
         <v>481</v>
@@ -13636,7 +13640,7 @@
         <v>204</v>
       </c>
       <c r="S192" s="6">
-        <v>180</v>
+        <v>222</v>
       </c>
       <c r="T192" s="2" t="s">
         <v>483</v>
@@ -13698,7 +13702,7 @@
         <v>245</v>
       </c>
       <c r="S193" s="6">
-        <v>181</v>
+        <v>267</v>
       </c>
       <c r="T193" s="2" t="s">
         <v>485</v>
@@ -13760,7 +13764,7 @@
         <v>246</v>
       </c>
       <c r="S194" s="6">
-        <v>182</v>
+        <v>268</v>
       </c>
       <c r="T194" s="2" t="s">
         <v>487</v>
@@ -13822,7 +13826,7 @@
         <v>247</v>
       </c>
       <c r="S195" s="6">
-        <v>183</v>
+        <v>269</v>
       </c>
       <c r="T195" s="2" t="s">
         <v>489</v>
@@ -13884,7 +13888,7 @@
         <v>248</v>
       </c>
       <c r="S196" s="6">
-        <v>184</v>
+        <v>270</v>
       </c>
       <c r="T196" s="2" t="s">
         <v>491</v>
@@ -13938,7 +13942,7 @@
         <v>29</v>
       </c>
       <c r="S197" s="6">
-        <v>186</v>
+        <v>33</v>
       </c>
       <c r="T197" s="2" t="s">
         <v>495</v>
@@ -13992,7 +13996,7 @@
         <v>30</v>
       </c>
       <c r="S198" s="6">
-        <v>187</v>
+        <v>34</v>
       </c>
       <c r="T198" s="2" t="s">
         <v>497</v>
@@ -14046,7 +14050,7 @@
         <v>31</v>
       </c>
       <c r="S199" s="6">
-        <v>188</v>
+        <v>35</v>
       </c>
       <c r="T199" s="2" t="s">
         <v>499</v>
@@ -14100,7 +14104,7 @@
         <v>32</v>
       </c>
       <c r="S200" s="6">
-        <v>189</v>
+        <v>36</v>
       </c>
       <c r="T200" s="2" t="s">
         <v>501</v>
@@ -14160,7 +14164,7 @@
         <v>73</v>
       </c>
       <c r="S201" s="6">
-        <v>190</v>
+        <v>81</v>
       </c>
       <c r="T201" s="2" t="s">
         <v>503</v>
@@ -14220,7 +14224,7 @@
         <v>74</v>
       </c>
       <c r="S202" s="6">
-        <v>191</v>
+        <v>82</v>
       </c>
       <c r="T202" s="2" t="s">
         <v>505</v>
@@ -14283,7 +14287,7 @@
         <v>75</v>
       </c>
       <c r="S203" s="6">
-        <v>192</v>
+        <v>83</v>
       </c>
       <c r="T203" s="2" t="s">
         <v>507</v>
@@ -14346,7 +14350,7 @@
         <v>76</v>
       </c>
       <c r="S204" s="6">
-        <v>193</v>
+        <v>84</v>
       </c>
       <c r="T204" s="2" t="s">
         <v>509</v>
@@ -14403,7 +14407,7 @@
         <v>117</v>
       </c>
       <c r="S205" s="6">
-        <v>194</v>
+        <v>128</v>
       </c>
       <c r="T205" s="2" t="s">
         <v>511</v>
@@ -14460,7 +14464,7 @@
         <v>118</v>
       </c>
       <c r="S206" s="6">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="T206" s="2" t="s">
         <v>513</v>
@@ -14517,7 +14521,7 @@
         <v>119</v>
       </c>
       <c r="S207" s="6">
-        <v>195</v>
+        <v>130</v>
       </c>
       <c r="T207" s="2" t="s">
         <v>515</v>
@@ -14574,7 +14578,7 @@
         <v>120</v>
       </c>
       <c r="S208" s="6">
-        <v>196</v>
+        <v>131</v>
       </c>
       <c r="T208" s="2" t="s">
         <v>517</v>
@@ -14637,7 +14641,7 @@
         <v>161</v>
       </c>
       <c r="S209" s="6">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="T209" s="2" t="s">
         <v>519</v>
@@ -14700,7 +14704,7 @@
         <v>162</v>
       </c>
       <c r="S210" s="6">
-        <v>199</v>
+        <v>177</v>
       </c>
       <c r="T210" s="2" t="s">
         <v>521</v>
@@ -14763,7 +14767,7 @@
         <v>163</v>
       </c>
       <c r="S211" s="6">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="T211" s="2" t="s">
         <v>523</v>
@@ -14826,7 +14830,7 @@
         <v>164</v>
       </c>
       <c r="S212" s="6">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="T212" s="2" t="s">
         <v>525</v>
@@ -14889,7 +14893,7 @@
         <v>205</v>
       </c>
       <c r="S213" s="6">
-        <v>202</v>
+        <v>224</v>
       </c>
       <c r="T213" s="2" t="s">
         <v>527</v>
@@ -14952,7 +14956,7 @@
         <v>206</v>
       </c>
       <c r="S214" s="6">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="T214" s="2" t="s">
         <v>529</v>
@@ -15015,7 +15019,7 @@
         <v>207</v>
       </c>
       <c r="S215" s="6">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="T215" s="2" t="s">
         <v>531</v>
@@ -15078,7 +15082,7 @@
         <v>208</v>
       </c>
       <c r="S216" s="6">
-        <v>205</v>
+        <v>227</v>
       </c>
       <c r="T216" s="2" t="s">
         <v>533</v>
@@ -15143,7 +15147,7 @@
         <v>249</v>
       </c>
       <c r="S217" s="6">
-        <v>206</v>
+        <v>271</v>
       </c>
       <c r="T217" s="2" t="s">
         <v>535</v>
@@ -15208,7 +15212,7 @@
         <v>250</v>
       </c>
       <c r="S218" s="6">
-        <v>207</v>
+        <v>272</v>
       </c>
       <c r="T218" s="2" t="s">
         <v>537</v>
@@ -15273,7 +15277,7 @@
         <v>251</v>
       </c>
       <c r="S219" s="6">
-        <v>208</v>
+        <v>273</v>
       </c>
       <c r="T219" s="2" t="s">
         <v>539</v>
@@ -15338,7 +15342,7 @@
         <v>252</v>
       </c>
       <c r="S220" s="6">
-        <v>209</v>
+        <v>274</v>
       </c>
       <c r="T220" s="2" t="s">
         <v>541</v>
@@ -15395,7 +15399,7 @@
         <v>33</v>
       </c>
       <c r="S221" s="6">
-        <v>211</v>
+        <v>37</v>
       </c>
       <c r="T221" s="2" t="s">
         <v>545</v>
@@ -15452,7 +15456,7 @@
         <v>34</v>
       </c>
       <c r="S222" s="6">
-        <v>212</v>
+        <v>38</v>
       </c>
       <c r="T222" s="2" t="s">
         <v>547</v>
@@ -15509,7 +15513,7 @@
         <v>35</v>
       </c>
       <c r="S223" s="6">
-        <v>213</v>
+        <v>39</v>
       </c>
       <c r="T223" s="2" t="s">
         <v>549</v>
@@ -15566,7 +15570,7 @@
         <v>36</v>
       </c>
       <c r="S224" s="6">
-        <v>214</v>
+        <v>40</v>
       </c>
       <c r="T224" s="2" t="s">
         <v>551</v>
@@ -15629,7 +15633,7 @@
         <v>77</v>
       </c>
       <c r="S225" s="6">
-        <v>215</v>
+        <v>85</v>
       </c>
       <c r="T225" s="2" t="s">
         <v>553</v>
@@ -15692,7 +15696,7 @@
         <v>78</v>
       </c>
       <c r="S226" s="6">
-        <v>216</v>
+        <v>86</v>
       </c>
       <c r="T226" s="2" t="s">
         <v>555</v>
@@ -15752,7 +15756,7 @@
         <v>79</v>
       </c>
       <c r="S227" s="6">
-        <v>217</v>
+        <v>87</v>
       </c>
       <c r="T227" s="2" t="s">
         <v>557</v>
@@ -15812,7 +15816,7 @@
         <v>80</v>
       </c>
       <c r="S228" s="6">
-        <v>218</v>
+        <v>88</v>
       </c>
       <c r="T228" s="2" t="s">
         <v>559</v>
@@ -15866,7 +15870,7 @@
         <v>121</v>
       </c>
       <c r="S229" s="6">
-        <v>219</v>
+        <v>133</v>
       </c>
       <c r="T229" s="2" t="s">
         <v>561</v>
@@ -15920,7 +15924,7 @@
         <v>122</v>
       </c>
       <c r="S230" s="6">
-        <v>220</v>
+        <v>134</v>
       </c>
       <c r="T230" s="2" t="s">
         <v>563</v>
@@ -15974,7 +15978,7 @@
         <v>123</v>
       </c>
       <c r="S231" s="6">
-        <v>221</v>
+        <v>135</v>
       </c>
       <c r="T231" s="2" t="s">
         <v>565</v>
@@ -16028,7 +16032,7 @@
         <v>124</v>
       </c>
       <c r="S232" s="6">
-        <v>222</v>
+        <v>136</v>
       </c>
       <c r="T232" s="2" t="s">
         <v>567</v>
@@ -16088,7 +16092,7 @@
         <v>165</v>
       </c>
       <c r="S233" s="6">
-        <v>224</v>
+        <v>180</v>
       </c>
       <c r="T233" s="2" t="s">
         <v>569</v>
@@ -16148,7 +16152,7 @@
         <v>166</v>
       </c>
       <c r="S234" s="6">
-        <v>225</v>
+        <v>181</v>
       </c>
       <c r="T234" s="2" t="s">
         <v>571</v>
@@ -16208,7 +16212,7 @@
         <v>167</v>
       </c>
       <c r="S235" s="6">
-        <v>226</v>
+        <v>182</v>
       </c>
       <c r="T235" s="2" t="s">
         <v>573</v>
@@ -16268,7 +16272,7 @@
         <v>168</v>
       </c>
       <c r="S236" s="6">
-        <v>227</v>
+        <v>183</v>
       </c>
       <c r="T236" s="2" t="s">
         <v>575</v>
@@ -16570,7 +16574,7 @@
         <v>253</v>
       </c>
       <c r="S241" s="6">
-        <v>232</v>
+        <v>276</v>
       </c>
       <c r="T241" s="2" t="s">
         <v>585</v>
@@ -16632,7 +16636,7 @@
         <v>254</v>
       </c>
       <c r="S242" s="6">
-        <v>233</v>
+        <v>277</v>
       </c>
       <c r="T242" s="2" t="s">
         <v>587</v>
@@ -16694,7 +16698,7 @@
         <v>255</v>
       </c>
       <c r="S243" s="6">
-        <v>234</v>
+        <v>278</v>
       </c>
       <c r="T243" s="2" t="s">
         <v>589</v>
@@ -16756,7 +16760,7 @@
         <v>256</v>
       </c>
       <c r="S244" s="6">
-        <v>235</v>
+        <v>279</v>
       </c>
       <c r="T244" s="2" t="s">
         <v>591</v>
@@ -16810,7 +16814,7 @@
         <v>37</v>
       </c>
       <c r="S245" s="6">
-        <v>237</v>
+        <v>42</v>
       </c>
       <c r="T245" s="2" t="s">
         <v>595</v>
@@ -16864,7 +16868,7 @@
         <v>38</v>
       </c>
       <c r="S246" s="6">
-        <v>238</v>
+        <v>43</v>
       </c>
       <c r="T246" s="2" t="s">
         <v>597</v>
@@ -16918,7 +16922,7 @@
         <v>39</v>
       </c>
       <c r="S247" s="6">
-        <v>239</v>
+        <v>44</v>
       </c>
       <c r="T247" s="2" t="s">
         <v>599</v>
@@ -16972,7 +16976,7 @@
         <v>40</v>
       </c>
       <c r="S248" s="6">
-        <v>240</v>
+        <v>45</v>
       </c>
       <c r="T248" s="2" t="s">
         <v>601</v>
@@ -17032,7 +17036,7 @@
         <v>81</v>
       </c>
       <c r="S249" s="6">
-        <v>241</v>
+        <v>89</v>
       </c>
       <c r="T249" s="2" t="s">
         <v>603</v>
@@ -17092,7 +17096,7 @@
         <v>82</v>
       </c>
       <c r="S250" s="6">
-        <v>242</v>
+        <v>90</v>
       </c>
       <c r="T250" s="2" t="s">
         <v>605</v>
@@ -17152,7 +17156,7 @@
         <v>83</v>
       </c>
       <c r="S251" s="6">
-        <v>243</v>
+        <v>91</v>
       </c>
       <c r="T251" s="2" t="s">
         <v>607</v>
@@ -17212,7 +17216,7 @@
         <v>84</v>
       </c>
       <c r="S252" s="6">
-        <v>244</v>
+        <v>92</v>
       </c>
       <c r="T252" s="2" t="s">
         <v>609</v>
@@ -17266,7 +17270,7 @@
         <v>125</v>
       </c>
       <c r="S253" s="6">
-        <v>245</v>
+        <v>137</v>
       </c>
       <c r="T253" s="2" t="s">
         <v>611</v>
@@ -17320,7 +17324,7 @@
         <v>126</v>
       </c>
       <c r="S254" s="6">
-        <v>246</v>
+        <v>138</v>
       </c>
       <c r="T254" s="2" t="s">
         <v>613</v>
@@ -17374,7 +17378,7 @@
         <v>127</v>
       </c>
       <c r="S255" s="6">
-        <v>247</v>
+        <v>139</v>
       </c>
       <c r="T255" s="2" t="s">
         <v>615</v>
@@ -17428,7 +17432,7 @@
         <v>128</v>
       </c>
       <c r="S256" s="6">
-        <v>248</v>
+        <v>140</v>
       </c>
       <c r="T256" s="2" t="s">
         <v>617</v>
@@ -17488,7 +17492,7 @@
         <v>169</v>
       </c>
       <c r="S257" s="6">
-        <v>250</v>
+        <v>185</v>
       </c>
       <c r="T257" s="2" t="s">
         <v>619</v>
@@ -17548,7 +17552,7 @@
         <v>170</v>
       </c>
       <c r="S258" s="6">
-        <v>251</v>
+        <v>186</v>
       </c>
       <c r="T258" s="2" t="s">
         <v>621</v>
@@ -17608,7 +17612,7 @@
         <v>171</v>
       </c>
       <c r="S259" s="6">
-        <v>252</v>
+        <v>187</v>
       </c>
       <c r="T259" s="2" t="s">
         <v>623</v>
@@ -17668,7 +17672,7 @@
         <v>172</v>
       </c>
       <c r="S260" s="6">
-        <v>253</v>
+        <v>188</v>
       </c>
       <c r="T260" s="2" t="s">
         <v>625</v>
@@ -17728,7 +17732,7 @@
         <v>213</v>
       </c>
       <c r="S261" s="6">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="T261" s="2" t="s">
         <v>627</v>
@@ -17788,7 +17792,7 @@
         <v>214</v>
       </c>
       <c r="S262" s="6">
-        <v>255</v>
+        <v>233</v>
       </c>
       <c r="T262" s="2" t="s">
         <v>629</v>
@@ -17848,7 +17852,7 @@
         <v>215</v>
       </c>
       <c r="S263" s="6">
-        <v>256</v>
+        <v>234</v>
       </c>
       <c r="T263" s="2" t="s">
         <v>631</v>
@@ -17908,7 +17912,7 @@
         <v>216</v>
       </c>
       <c r="S264" s="6">
-        <v>257</v>
+        <v>235</v>
       </c>
       <c r="T264" s="2" t="s">
         <v>633</v>
@@ -17970,7 +17974,7 @@
         <v>257</v>
       </c>
       <c r="S265" s="6">
-        <v>258</v>
+        <v>280</v>
       </c>
       <c r="T265" s="2" t="s">
         <v>635</v>
@@ -18032,7 +18036,7 @@
         <v>258</v>
       </c>
       <c r="S266" s="6">
-        <v>259</v>
+        <v>281</v>
       </c>
       <c r="T266" s="2" t="s">
         <v>637</v>
@@ -18094,7 +18098,7 @@
         <v>259</v>
       </c>
       <c r="S267" s="6">
-        <v>260</v>
+        <v>282</v>
       </c>
       <c r="T267" s="2" t="s">
         <v>639</v>
@@ -18156,7 +18160,7 @@
         <v>260</v>
       </c>
       <c r="S268" s="6">
-        <v>261</v>
+        <v>283</v>
       </c>
       <c r="T268" s="2" t="s">
         <v>641</v>
@@ -18210,7 +18214,7 @@
         <v>41</v>
       </c>
       <c r="S269" s="6">
-        <v>263</v>
+        <v>46</v>
       </c>
       <c r="T269" s="2" t="s">
         <v>645</v>
@@ -18264,7 +18268,7 @@
         <v>42</v>
       </c>
       <c r="S270" s="6">
-        <v>264</v>
+        <v>47</v>
       </c>
       <c r="T270" s="2" t="s">
         <v>647</v>
@@ -18318,7 +18322,7 @@
         <v>43</v>
       </c>
       <c r="S271" s="6">
-        <v>265</v>
+        <v>48</v>
       </c>
       <c r="T271" s="2" t="s">
         <v>649</v>
@@ -18372,7 +18376,7 @@
         <v>44</v>
       </c>
       <c r="S272" s="6">
-        <v>266</v>
+        <v>49</v>
       </c>
       <c r="T272" s="2" t="s">
         <v>651</v>
@@ -18432,7 +18436,7 @@
         <v>85</v>
       </c>
       <c r="S273" s="6">
-        <v>267</v>
+        <v>94</v>
       </c>
       <c r="T273" s="2" t="s">
         <v>653</v>
@@ -18492,7 +18496,7 @@
         <v>86</v>
       </c>
       <c r="S274" s="6">
-        <v>268</v>
+        <v>95</v>
       </c>
       <c r="T274" s="2" t="s">
         <v>655</v>
@@ -18552,7 +18556,7 @@
         <v>87</v>
       </c>
       <c r="S275" s="6">
-        <v>269</v>
+        <v>96</v>
       </c>
       <c r="T275" s="2" t="s">
         <v>657</v>
@@ -18612,7 +18616,7 @@
         <v>88</v>
       </c>
       <c r="S276" s="6">
-        <v>270</v>
+        <v>97</v>
       </c>
       <c r="T276" s="2" t="s">
         <v>659</v>
@@ -18666,7 +18670,7 @@
         <v>129</v>
       </c>
       <c r="S277" s="6">
-        <v>271</v>
+        <v>141</v>
       </c>
       <c r="T277" s="2" t="s">
         <v>661</v>
@@ -18720,7 +18724,7 @@
         <v>130</v>
       </c>
       <c r="S278" s="6">
-        <v>272</v>
+        <v>142</v>
       </c>
       <c r="T278" s="2" t="s">
         <v>663</v>
@@ -18774,7 +18778,7 @@
         <v>131</v>
       </c>
       <c r="S279" s="6">
-        <v>273</v>
+        <v>143</v>
       </c>
       <c r="T279" s="2" t="s">
         <v>665</v>
@@ -18828,7 +18832,7 @@
         <v>132</v>
       </c>
       <c r="S280" s="6">
-        <v>274</v>
+        <v>144</v>
       </c>
       <c r="T280" s="2" t="s">
         <v>667</v>
@@ -18888,7 +18892,7 @@
         <v>173</v>
       </c>
       <c r="S281" s="6">
-        <v>276</v>
+        <v>189</v>
       </c>
       <c r="T281" s="2" t="s">
         <v>669</v>
@@ -18948,7 +18952,7 @@
         <v>174</v>
       </c>
       <c r="S282" s="6">
-        <v>277</v>
+        <v>190</v>
       </c>
       <c r="T282" s="2" t="s">
         <v>671</v>
@@ -19008,7 +19012,7 @@
         <v>175</v>
       </c>
       <c r="S283" s="6">
-        <v>278</v>
+        <v>191</v>
       </c>
       <c r="T283" s="2" t="s">
         <v>673</v>
@@ -19068,7 +19072,7 @@
         <v>176</v>
       </c>
       <c r="S284" s="6">
-        <v>279</v>
+        <v>192</v>
       </c>
       <c r="T284" s="2" t="s">
         <v>675</v>
@@ -19128,7 +19132,7 @@
         <v>217</v>
       </c>
       <c r="S285" s="6">
-        <v>280</v>
+        <v>237</v>
       </c>
       <c r="T285" s="2" t="s">
         <v>677</v>
@@ -19188,7 +19192,7 @@
         <v>218</v>
       </c>
       <c r="S286" s="6">
-        <v>281</v>
+        <v>238</v>
       </c>
       <c r="T286" s="2" t="s">
         <v>679</v>
@@ -19248,7 +19252,7 @@
         <v>219</v>
       </c>
       <c r="S287" s="6">
-        <v>282</v>
+        <v>239</v>
       </c>
       <c r="T287" s="2" t="s">
         <v>681</v>
@@ -19308,7 +19312,7 @@
         <v>220</v>
       </c>
       <c r="S288" s="6">
-        <v>283</v>
+        <v>240</v>
       </c>
       <c r="T288" s="2" t="s">
         <v>683</v>

</xml_diff>